<commit_message>
Connected Core düzeltmeleri + Fortress Core + hikaye dosyası
- game_scene.gd: _get_ball_core_type inner_core_type döndürüyor (UI sprite fix)
- game_scene.gd: _CORE_FOLDER_MAP'e tüm Connected Core klasörleri eklendi
- game_scene.gd: _CORE_INDEX_MAP'e Vector Connected Core index'leri (180-184) eklendi
- game_scene.gd: _CONNECTED_CORE_INDICES const + kart UI'da Connected Core badge
- player.gd: INNER_ORBIT_RADIUS 35 → 65 (eski dış orbit boyutunda)
- player.gd: add_to_orbit Connected Core'lara scale=1.0, orbit toplarına scale=0
- ball.gd: Fortress Core sürekli çalışır (timer bağımsız), tüm düşmanlara uygular
- vectorCards.xlsx: Fortress Core açıklaması güncellendi
- stority.txt: Oyun hikayesi eklendi
</commit_message>
<xml_diff>
--- a/vectorCards.xlsx
+++ b/vectorCards.xlsx
@@ -924,12 +924,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Armor %75+ doluyken: | 90px düşmanlar %25 yavaşlar</t>
+          <t>Armor %75+ doluyken: 90px icindeki tum dusmanlara surekli %25 yavaslatma uygular</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Zırh %75+: 90px yavaşlatma %25 (1s)</t>
+          <t>Armor %75+: 90px'e surekli %25 yavaslatma</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">

</xml_diff>